<commit_message>
Add 7 new companies 2026-09-11
</commit_message>
<xml_diff>
--- a/master_companies.xlsx
+++ b/master_companies.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3221,10 +3221,8 @@
           <t>https://niro360.co.il/</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>0260409</t>
-        </is>
+      <c r="F98" t="n">
+        <v>260409</v>
       </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
@@ -3248,10 +3246,8 @@
           <t>https://greenbook.co.il/card/7644/19000</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>0503977046</t>
-        </is>
+      <c r="F99" t="n">
+        <v>503977046</v>
       </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr"/>
@@ -3275,10 +3271,8 @@
           <t>https://eden-or.zapweb.co.il/</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>0737533575</t>
-        </is>
+      <c r="F100" t="n">
+        <v>737533575</v>
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
@@ -3302,14 +3296,217 @@
           <t>https://www.calcalit-yeruham.co.il/product/2649</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>089201208</t>
-        </is>
+      <c r="F101" t="n">
+        <v>89201208</v>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr"/>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>ניהול נכסים בירושלים | חברת אחזקה וניקיון בירושלים - שמדר</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>ירושלים</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>mshamdar@gmail.com</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>http://shamdar-management.co.il/</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>0774040881</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr"/>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>קבוצת אשד – ניהול פרויקטים רחבי היקף בתחומי הנדל"ן, הנדסה ותפעול</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>חולון</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>eshed-m@eshed-m.co.il</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>https://www.eshed-m.co.il/</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>035386666</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr"/>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>ERB Proximo: שירותי CFO לחברות סטארטאפ והייטק הפועלות בארה ...</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>אשקלון</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>info@erb.co.il</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>https://www.erb.co.il/</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>0260520</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr"/>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>חברת החשמל לישראל בעמ</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>אשקלון</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>valeriia.kuznetsova@spglobal.com</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>https://www.maalot.co.il/Entity/Index/1482</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>037539742</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr"/>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>מכרזי ספקים - החברה הכלכלית בלוד</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>yasminb@calcalitlod.co.il</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>https://calcalitlod.co.il/%D7%9E%D7%9B%D7%A8%D7%96%D7%99-%D7%A1%D7%A4%D7%A7%D7%99%D7%9D/</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>0210628</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr"/>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>מכרז למתן שירותי ניהול פרויקט, תיאום ופיקוח בישוב מעלה אדומים</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>yaakova@moch.gov.il</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>https://mr.gov.il/ilgstorefront/he/p/508580</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>0920201036</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr"/>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>אודות</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Info@r-projects.co.il</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>https://www.r-projects.co.il/About</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>0779707479</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 13 new companies 2026-09-18
</commit_message>
<xml_diff>
--- a/master_companies.xlsx
+++ b/master_companies.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3325,10 +3325,8 @@
           <t>http://shamdar-management.co.il/</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>0774040881</t>
-        </is>
+      <c r="F102" t="n">
+        <v>774040881</v>
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr"/>
@@ -3356,10 +3354,8 @@
           <t>https://www.eshed-m.co.il/</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>035386666</t>
-        </is>
+      <c r="F103" t="n">
+        <v>35386666</v>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
@@ -3387,10 +3383,8 @@
           <t>https://www.erb.co.il/</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>0260520</t>
-        </is>
+      <c r="F104" t="n">
+        <v>260520</v>
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr"/>
@@ -3418,10 +3412,8 @@
           <t>https://www.maalot.co.il/Entity/Index/1482</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>037539742</t>
-        </is>
+      <c r="F105" t="n">
+        <v>37539742</v>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
@@ -3445,10 +3437,8 @@
           <t>https://calcalitlod.co.il/%D7%9E%D7%9B%D7%A8%D7%96%D7%99-%D7%A1%D7%A4%D7%A7%D7%99%D7%9D/</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>0210628</t>
-        </is>
+      <c r="F106" t="n">
+        <v>210628</v>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr"/>
@@ -3472,10 +3462,8 @@
           <t>https://mr.gov.il/ilgstorefront/he/p/508580</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>0920201036</t>
-        </is>
+      <c r="F107" t="n">
+        <v>920201036</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
@@ -3499,14 +3487,387 @@
           <t>https://www.r-projects.co.il/About</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>0779707479</t>
-        </is>
+      <c r="F108" t="n">
+        <v>779707479</v>
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr"/>
       <c r="I108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr"/>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>דקהדאנס 2026</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>באר שבע</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>batsheva@batsheva.co.il</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>https://batsheva.co.il/repertory/%D7%93%D7%A7%D7%94%D7%93%D7%90%D7%A0%D7%A1-2025/</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>0260831</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr"/>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>ידידי בת־שבע בישראל</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>באר שבע</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>israelifriends@batsheva.co.il</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>https://batsheva.co.il/israel_friends/</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>0260824</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr"/>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>סניף באר שבע</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>באר שבע</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>snif_beer7@cancer.org.il</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>https://www.cancer.org.il/branches/regions/south/</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>00599995</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr"/>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>ת"י ISO 9001 - מערכת ניהול איכות</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>כפר סבא</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>avital_w@sii.org.il</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>https://www.sii.org.il/he/lobby/qualityauth/quality-management-systems/iso-9001</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>022549090</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr"/>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>קבוצת CPM - ניהול פרויקטים בבנייה - תכנון פרויקטים, יזמות נדל"ן מניב</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>מודיעין</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>office@www.cpm.co.il</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>https://www.cpm.co.il/</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>03070308</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr"/>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>גזברות - מחוז אשקלון | משרד הבריאות</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>אשקלון</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>gizbarutlba@bmc.gov.il</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>https://www.gov.il/he/government-service-branches/moh-ashkelon-finance-n</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>086745306</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr"/>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>תורת ניהול היער בישראל - קרן קימת לישראל - קק"ל</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr"/>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>pneyot-tzibur@kkl.org.il</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>https://www.kkl.org.il/forest_management_principles/</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>0755111393</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr"/>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>עמיגור: עמוד הבית</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr"/>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>moked@amigour.co.il</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>https://www.amigour.co.il/</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>0260914</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr"/>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>שירותי ניהול</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr"/>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>israel@d-zefat.com</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>https://diamondsalley.co.il/%D7%A9%D7%99%D7%A8%D7%95%D7%AA%D7%99-%D7%A0%D7%99%D7%94%D7%95%D7%9C/</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>0260901</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr"/>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>דו"חות ופרסומי המועצה</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr"/>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>liat@telerom.co.il</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>https://www.zy1882.co.il/FileDownloads/?nodeId=1052</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>057229204772</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr"/>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>מצפה "אביב של העמק"</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr"/>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>team@giveback.co.il</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>https://giveback.co.il/project/88943</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>0260702</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr"/>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>קָמָה ניהול ואחזקת נכסים: ניהול נדל"ן עסקי ופרטי</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr"/>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>info@kamanagement.co.il</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>https://kamanagement.co.il/</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>076458117215</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr"/>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>בר-און - ניהול נכסים</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr"/>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>office@bar-onmanage.co.il</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>https://bar-onmanage.co.il/</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>0250827</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 35 new companies 2026-09-25
</commit_message>
<xml_diff>
--- a/master_companies.xlsx
+++ b/master_companies.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I121"/>
+  <dimension ref="A1:I156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3516,10 +3516,8 @@
           <t>https://batsheva.co.il/repertory/%D7%93%D7%A7%D7%94%D7%93%D7%90%D7%A0%D7%A1-2025/</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>0260831</t>
-        </is>
+      <c r="F109" t="n">
+        <v>260831</v>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
@@ -3547,10 +3545,8 @@
           <t>https://batsheva.co.il/israel_friends/</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>0260824</t>
-        </is>
+      <c r="F110" t="n">
+        <v>260824</v>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr"/>
@@ -3578,10 +3574,8 @@
           <t>https://www.cancer.org.il/branches/regions/south/</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>00599995</t>
-        </is>
+      <c r="F111" t="n">
+        <v>599995</v>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
@@ -3609,10 +3603,8 @@
           <t>https://www.sii.org.il/he/lobby/qualityauth/quality-management-systems/iso-9001</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>022549090</t>
-        </is>
+      <c r="F112" t="n">
+        <v>22549090</v>
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr"/>
@@ -3640,10 +3632,8 @@
           <t>https://www.cpm.co.il/</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>03070308</t>
-        </is>
+      <c r="F113" t="n">
+        <v>3070308</v>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
@@ -3671,10 +3661,8 @@
           <t>https://www.gov.il/he/government-service-branches/moh-ashkelon-finance-n</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>086745306</t>
-        </is>
+      <c r="F114" t="n">
+        <v>86745306</v>
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr"/>
@@ -3698,10 +3686,8 @@
           <t>https://www.kkl.org.il/forest_management_principles/</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>0755111393</t>
-        </is>
+      <c r="F115" t="n">
+        <v>755111393</v>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
@@ -3725,10 +3711,8 @@
           <t>https://www.amigour.co.il/</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>0260914</t>
-        </is>
+      <c r="F116" t="n">
+        <v>260914</v>
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr"/>
@@ -3752,10 +3736,8 @@
           <t>https://diamondsalley.co.il/%D7%A9%D7%99%D7%A8%D7%95%D7%AA%D7%99-%D7%A0%D7%99%D7%94%D7%95%D7%9C/</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>0260901</t>
-        </is>
+      <c r="F117" t="n">
+        <v>260901</v>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
@@ -3779,10 +3761,8 @@
           <t>https://www.zy1882.co.il/FileDownloads/?nodeId=1052</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>057229204772</t>
-        </is>
+      <c r="F118" t="n">
+        <v>57229204772</v>
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr"/>
@@ -3806,10 +3786,8 @@
           <t>https://giveback.co.il/project/88943</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>0260702</t>
-        </is>
+      <c r="F119" t="n">
+        <v>260702</v>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
@@ -3833,10 +3811,8 @@
           <t>https://kamanagement.co.il/</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>076458117215</t>
-        </is>
+      <c r="F120" t="n">
+        <v>76458117215</v>
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr"/>
@@ -3860,14 +3836,981 @@
           <t>https://bar-onmanage.co.il/</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>0250827</t>
-        </is>
+      <c r="F121" t="n">
+        <v>250827</v>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr"/>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>חברת ניהול בתל אביב - קצר ולעניין-072-392-1774</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>תל אביב</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>yinon@short-point.com</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>https://www.short-point.co.il/%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91%D7%AA%D7%9C-%D7%90%D7%91%D7%99%D7%91/</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>0723921774</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr"/>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>ניהול נכסים בתל אביב</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>תל אביב</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>office@delacasa.co.il</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>https://delacasa.co.il/%D7%A4%D7%A8%D7%95%D7%99%D7%99%D7%A7%D7%98/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%91%D7%AA%D7%9C-%D7%90%D7%91%D7%99%D7%91/</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>0230420</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr"/>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>אחזקת דירות ברמת גן | שירות לבעלי נכסים</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>רמת גן</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>micky@housemanager.co.il</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>https://www.housemanager.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%91%D7%A8%D7%9E%D7%AA-%D7%92%D7%9F/</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>0220725</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr"/>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>מעל כולן: נבחרה חברת התעופה הכי טובה בעולם</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>חולון</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>info@mako.co.il</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>https://www.mako.co.il/travel-news/israel/Article-20fa2d1558db0a1027.htm</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>000005201000</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr"/>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>אדן ניהול בתים משותפים</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>בת ים</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>nadav@edenbatim.com</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>https://www.kehilot.co.il/company/%D7%90%D7%93%D7%9F-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91%D7%AA%D7%99%D7%9D-%D7%9E%D7%A9%D7%95%D7%AA%D7%A4%D7%99%D7%9D/</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>0260816</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr"/>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>חברת ניהול</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>מודיעין</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>info@mei-modiin.co.il</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>https://mei-modiin.co.il/index.php?option=com_content&amp;view=article&amp;id=387:%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C&amp;catid=105</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>00300420</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr"/>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>עורך דין ניהול מו״מ מול קבלנים בקריית שמונה</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr"/>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>office@ofirchen-law.co.il</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>https://ofirchen-law.co.il/LocalLanding?serviceId=seed-svc-company-liquidation&amp;subService=%D7%A0%D7%99%D7%94%D7%95%D7%9C%20%D7%9E%D7%95%D7%B4%D7%9E%20%D7%9E%D7%95%D7%9C%20%D7%A7%D7%91%D7%9C%D7%A0%D7%99%D7%9D&amp;city=%D7%A7%D7%A8%D7%99%D7%99%D7%AA%20%D7%A9%D7%9E%D7%95%D7%A0%D7%94</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>0547864802</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr"/>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>רהט</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr"/>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>pniot@ankori.co.il</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>https://www.theorytest.org.il/branches/%D7%A8%D7%94%D7%98/</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>0241105</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr"/>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>גדעון רהט - המחלקה למדע המדינה</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>ירושלים</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>msgrah@mail.huji.ac.il</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>https://politics.huji.ac.il/people/%D7%93%D7%9F-%D7%90%D7%91%D7%A0%D7%95%D7%9F</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>025881116</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr"/>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>ניהול תיק רפואי ע"י אחות באום אל-פחם - מומלצים</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr"/>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>info@medreviews.co.il</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>https://www.medreviews.co.il/search/treatment/medical-management-by-nurse/north/umm-al-fahm</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>0554548554</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr"/>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>כרמיאל | Page 26</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr"/>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>pniot@mwg.org.il</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>https://www.mwg.org.il/he/%D7%9E%D7%95%D7%A2%D7%A6%D7%94%D7%90%D7%96%D7%95%D7%A8/%D7%9B%D7%A8%D7%9E%D7%99%D7%90%D7%9C?page=25</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>044189881257</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr"/>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>ניהול נכסים בגבעתיים</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr"/>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>info@caesar.co.il</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>https://www.caesar.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%91%D7%92%D7%91%D7%A2%D7%AA%D7%99%D7%99%D7%9D-%D7%94%D7%97%D7%91%D7%A8%D7%94-%D7%94%D7%9E%D7%95%D7%9E%D7%9C%D7%A6%D7%AA-%D7%9C%D7%A0/</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>0525416313</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr"/>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>אתהל | ניהול ואחזקת מבנים: ראשי</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>e.atahel@gmail.com</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>https://atahel.co.il/</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>0260224</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr"/>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>עורך דין ניהול מו״מ מול קבלנים במעלה אדומים</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr"/>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>office@ofirchen-law.co.il</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>https://www.ofirchen-law.co.il/LocalLanding?city=%D7%9E%D7%A2%D7%9C%D7%94+%D7%90%D7%93%D7%95%D7%9E%D7%99%D7%9D&amp;serviceId=69334252d53ee94fc5dc57b8&amp;subService=%D7%A0%D7%99%D7%94%D7%95%D7%9C+%D7%9E%D7%95%D7%B4%D7%9E+%D7%9E%D7%95%D7%9C+%D7%A7%D7%91%D7%9C%D7%A0%D7%99%D7%9D</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>0547864802</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr"/>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>מה אתה עושה בחיים אלעד הדר</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr"/>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>20elad@bizsuccess.co.il</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>https://bizsuccess.co.il/%D7%9E%D7%94-%D7%90%D7%AA%D7%94-%D7%A2%D7%95%D7%A9%D7%94-%D7%91%D7%97%D7%99%D7%99%D7%9D-%D7%90%D7%9C%D7%A2%D7%93-%D7%94%D7%93%D7%A8/?srsltid=AU7gw4WXOjq3WQM4Su8fXK_EPoNk0tx8JzLm41-LBfhUzGfyL3rG9lWn</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>0260505</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr"/>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>חוגיםג'אז | מרכז קהילתי ראש העין</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr"/>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Sherut@levrh.org</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>http://makombalev.org.il/html5/dbMATENASIM.taf?DID=4469&amp;_0=%E2'%E0%E6</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>0524539151</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr"/>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>יהלום ניהול ואחזקה כפר יונה | ניהול בתים משותפים</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr"/>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>contact@nons.co.il</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>https://nons.co.il/provider/%D7%99%D7%94%D7%9C%D7%95%D7%9D_%D7%A0%D7%99%D7%94%D7%95%D7%9C_%D7%95%D7%90%D7%97%D7%96%D7%A7%D7%94</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>0509870040</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr"/>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>ניהול תיק רפואי ע"י אחות בכפר יונה - מומלצים</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr"/>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>info@medreviews.co.il</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>https://www.medreviews.co.il/search/treatment/medical-management-by-nurse/sharon/kfar-yona</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>0554548554</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr"/>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>אורי יעקב - אגף משאבי אנוש</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>uriya@savion.huji.ac.il</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>https://hr.huji.ac.il/people/%D7%90%D7%95%D7%A8%D7%99-%D7%99%D7%A2%D7%A7%D7%91</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>025881085</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr"/>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>יעקב ברנט - הרצוג עורכי דין</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr"/>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>contact@herzoglaw.co.il</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>https://herzoglaw.co.il/he/our-team/yaakov-brandt/</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>0260713</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr"/>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>עורך דין ניידות בסח'נין מומלץ לתביעות קצבת ניידות ביטוח לאומי</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr"/>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Mail@mt-law.co.il</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>https://www.mt-law.co.il/local/%D7%A2%D7%95%D7%A8%D7%9A-%D7%93%D7%99%D7%9F-%D7%A0%D7%99%D7%99%D7%93%D7%95%D7%AA-%D7%A1%D7%97%D7%A0%D7%99%D7%9F/</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>0260326</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr"/>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>חברת ניהול פרויקטים הנדסיים מגייסת מנכ״ל.ית</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr"/>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>info@connectedbusinesses.co.il</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>https://www.connectedbusinesses.co.il/job-offer/%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A4%D7%A8%D7%95%D7%99%D7%A7%D7%98%D7%99%D7%9D-%D7%94%D7%A0%D7%93%D7%A1%D7%99%D7%99%D7%9D-%D7%9E%D7%92%D7%99%D7%99%D7%A1%D7%AA-%D7%9E%D7%A0/</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>0260616</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr"/>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>חברה למימוש זכויות: ניהול וייעוץ מקצועי לזכויותיכם - תג חניה לנכה</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr"/>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>yakov@ybay.co.il</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>https://parkingtag.co.il/%D7%97%D7%91%D7%A8%D7%94-%D7%9C%D7%9E%D7%99%D7%9E%D7%95%D7%A9-%D7%96%D7%9B%D7%95%D7%99%D7%95%D7%AA/</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>0240814</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr"/>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>אופקים – חברה מנהלת להקמה ופיתוח שכונת הפארק, 1415 יחידות ...</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr"/>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>office@enp.co.il</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>https://enp.co.il/projects/%D7%90%D7%95%D7%A4%D7%A7%D7%99%D7%9D-%D7%97%D7%91%D7%A8%D7%94-%D7%9E%D7%A0%D7%94%D7%9C%D7%AA-%D7%9C%D7%94%D7%A7%D7%9E%D7%94-%D7%95%D7%A4%D7%99%D7%AA%D7%95%D7%97-%D7%A9%D7%9B%D7%95%D7%A0%D7%AA-%D7%94/</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>00021024</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr"/>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>אופקים | Page 2</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr"/>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>maavarim@merhavim.matnasim.co.il</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>https://www.mem.org.il/he/%D7%9E%D7%95%D7%A2%D7%A6%D7%94%D7%90%D7%96%D7%95%D7%A8/%D7%90%D7%95%D7%A4%D7%A7%D7%99%D7%9D?page=1</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>064266895223</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr"/>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>חברת ניהול בניינים קטנים – פתרון חכם לניהול בניינים משותפים - הדר אחזקות</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr"/>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Office.itayhadar@gmail.com</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>https://hadar-group.co.il/%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91%D7%A0%D7%99%D7%99%D7%A0%D7%99%D7%9D-%D7%A7%D7%98%D7%A0%D7%99%D7%9D-%D7%A4%D7%AA%D7%A8%D7%95%D7%9F-%D7%97%D7%9B%D7%9D-%D7%9C/</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>0260318</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr"/>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>אחזקת מבנים, ניקיון ואבטחה - סטנלי פרייס</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>wyosiw@gmail.com</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>https://architecture.org.il/%D7%90%D7%99%D7%A0%D7%93%D7%A7%D7%A1/%D7%90%D7%97%D7%96%D7%A7%D7%AA-%D7%9E%D7%91%D7%A0%D7%99%D7%9D-%D7%A0%D7%99%D7%A7%D7%99%D7%95%D7%9F-%D7%95%D7%90%D7%91%D7%98%D7%97%D7%94-%D7%A1%D7%98%D7%A0%D7%9C%D7%99-%D7%A4%D7%A8%D7%99%D7%99%D7%A1/</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>0250417</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr"/>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>7 דברים לבדוק לפני שבוחרים חברת ניהול ועד בית חיצונית</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr"/>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>office@centerteam.co.il</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>https://www.centerteam.co.il/7-%D7%93%D7%91%D7%A8%D7%99%D7%9D-%D7%9C%D7%91%D7%93%D7%95%D7%A7-%D7%9C%D7%A4%D7%A0%D7%99-%D7%A9%D7%91%D7%95%D7%97%D7%A8%D7%99%D7%9D-%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%95%D7%A2/</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>0260224</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr"/>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>צור קשר מנהל</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>michals@kaye.ac.il</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>https://kaye.ac.il/%D7%9E%D7%A0%D7%94%D7%9C-%D7%94%D7%A1%D7%98%D7%95%D7%93%D7%A0%D7%98%D7%99%D7%9D/%D7%A6%D7%95%D7%A8-%D7%A7%D7%A9%D7%A8/</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr"/>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>אגף מנהל תלמידים – אתך לאורך כל הדרך</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>eofier@univ.haifa.ac.il</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>https://mt.haifa.ac.il/</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>048288126</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr"/>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>חברת ניהול מבנים – כל המידע על השירות</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>info@rbsec.co.il</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>https://www.rbsec.co.il/%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%9E%D7%91%D7%A0%D7%99%D7%9D</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>035618888</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr"/>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>ניהול נכסים לרילוקיישן – פתרונות למשכירים ושוכרים</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>sales@ocean-il.co.il</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>https://www.ocean-il.co.il/%D7%A9%D7%99%D7%A8%D7%95%D7%AA%D7%99-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%9E%D7%94%D7%90%D7%A8%D7%A5-%D7%95%D7%9E%D7%A8%D7%97%D7%95%D7%A7/</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>010192625</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr"/>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>ניהול נכסים: כל מה שצריך לדעת</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Office@kfgroup.co.il</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>https://kfgroup.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%9B%D7%9C-%D7%9E%D7%94-%D7%A9%D7%A6%D7%A8%D7%99%D7%9A-%D7%9C%D7%93%D7%A2%D7%AA/</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>0240827</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr"/>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>אודות חברת מבנים</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr"/>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>office@bedek-mivnim.co.il</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>https://www.bedek-mivnim.co.il/%D7%90%D7%95%D7%93%D7%95%D7%AA.html</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>071899861</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr"/>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>מבנים רשת תיווך בקריות – תיווך מבנים עוסקת בהשכרה ובטיפול שנתי ...</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>mivnim2011@gmail.com</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>https://mivnim.co.il/</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>000040276453</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 6 new companies 2026-10-02
</commit_message>
<xml_diff>
--- a/master_companies.xlsx
+++ b/master_companies.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I156"/>
+  <dimension ref="A1:I162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3865,10 +3865,8 @@
           <t>https://www.short-point.co.il/%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91%D7%AA%D7%9C-%D7%90%D7%91%D7%99%D7%91/</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>0723921774</t>
-        </is>
+      <c r="F122" t="n">
+        <v>723921774</v>
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr"/>
@@ -3896,10 +3894,8 @@
           <t>https://delacasa.co.il/%D7%A4%D7%A8%D7%95%D7%99%D7%99%D7%A7%D7%98/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%91%D7%AA%D7%9C-%D7%90%D7%91%D7%99%D7%91/</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>0230420</t>
-        </is>
+      <c r="F123" t="n">
+        <v>230420</v>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr"/>
@@ -3927,10 +3923,8 @@
           <t>https://www.housemanager.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%91%D7%A8%D7%9E%D7%AA-%D7%92%D7%9F/</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>0220725</t>
-        </is>
+      <c r="F124" t="n">
+        <v>220725</v>
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr"/>
@@ -3958,10 +3952,8 @@
           <t>https://www.mako.co.il/travel-news/israel/Article-20fa2d1558db0a1027.htm</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>000005201000</t>
-        </is>
+      <c r="F125" t="n">
+        <v>5201000</v>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
@@ -3989,10 +3981,8 @@
           <t>https://www.kehilot.co.il/company/%D7%90%D7%93%D7%9F-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91%D7%AA%D7%99%D7%9D-%D7%9E%D7%A9%D7%95%D7%AA%D7%A4%D7%99%D7%9D/</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>0260816</t>
-        </is>
+      <c r="F126" t="n">
+        <v>260816</v>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr"/>
@@ -4020,10 +4010,8 @@
           <t>https://mei-modiin.co.il/index.php?option=com_content&amp;view=article&amp;id=387:%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C&amp;catid=105</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>00300420</t>
-        </is>
+      <c r="F127" t="n">
+        <v>300420</v>
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr"/>
@@ -4047,10 +4035,8 @@
           <t>https://ofirchen-law.co.il/LocalLanding?serviceId=seed-svc-company-liquidation&amp;subService=%D7%A0%D7%99%D7%94%D7%95%D7%9C%20%D7%9E%D7%95%D7%B4%D7%9E%20%D7%9E%D7%95%D7%9C%20%D7%A7%D7%91%D7%9C%D7%A0%D7%99%D7%9D&amp;city=%D7%A7%D7%A8%D7%99%D7%99%D7%AA%20%D7%A9%D7%9E%D7%95%D7%A0%D7%94</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>0547864802</t>
-        </is>
+      <c r="F128" t="n">
+        <v>547864802</v>
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr"/>
@@ -4074,10 +4060,8 @@
           <t>https://www.theorytest.org.il/branches/%D7%A8%D7%94%D7%98/</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>0241105</t>
-        </is>
+      <c r="F129" t="n">
+        <v>241105</v>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
@@ -4105,10 +4089,8 @@
           <t>https://politics.huji.ac.il/people/%D7%93%D7%9F-%D7%90%D7%91%D7%A0%D7%95%D7%9F</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>025881116</t>
-        </is>
+      <c r="F130" t="n">
+        <v>25881116</v>
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr"/>
@@ -4132,10 +4114,8 @@
           <t>https://www.medreviews.co.il/search/treatment/medical-management-by-nurse/north/umm-al-fahm</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>0554548554</t>
-        </is>
+      <c r="F131" t="n">
+        <v>554548554</v>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
@@ -4159,10 +4139,8 @@
           <t>https://www.mwg.org.il/he/%D7%9E%D7%95%D7%A2%D7%A6%D7%94%D7%90%D7%96%D7%95%D7%A8/%D7%9B%D7%A8%D7%9E%D7%99%D7%90%D7%9C?page=25</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr">
-        <is>
-          <t>044189881257</t>
-        </is>
+      <c r="F132" t="n">
+        <v>44189881257</v>
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr"/>
@@ -4186,10 +4164,8 @@
           <t>https://www.caesar.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%91%D7%92%D7%91%D7%A2%D7%AA%D7%99%D7%99%D7%9D-%D7%94%D7%97%D7%91%D7%A8%D7%94-%D7%94%D7%9E%D7%95%D7%9E%D7%9C%D7%A6%D7%AA-%D7%9C%D7%A0/</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>0525416313</t>
-        </is>
+      <c r="F133" t="n">
+        <v>525416313</v>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr"/>
@@ -4213,10 +4189,8 @@
           <t>https://atahel.co.il/</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr">
-        <is>
-          <t>0260224</t>
-        </is>
+      <c r="F134" t="n">
+        <v>260224</v>
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr"/>
@@ -4240,10 +4214,8 @@
           <t>https://www.ofirchen-law.co.il/LocalLanding?city=%D7%9E%D7%A2%D7%9C%D7%94+%D7%90%D7%93%D7%95%D7%9E%D7%99%D7%9D&amp;serviceId=69334252d53ee94fc5dc57b8&amp;subService=%D7%A0%D7%99%D7%94%D7%95%D7%9C+%D7%9E%D7%95%D7%B4%D7%9E+%D7%9E%D7%95%D7%9C+%D7%A7%D7%91%D7%9C%D7%A0%D7%99%D7%9D</t>
         </is>
       </c>
-      <c r="F135" t="inlineStr">
-        <is>
-          <t>0547864802</t>
-        </is>
+      <c r="F135" t="n">
+        <v>547864802</v>
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr"/>
@@ -4267,10 +4239,8 @@
           <t>https://bizsuccess.co.il/%D7%9E%D7%94-%D7%90%D7%AA%D7%94-%D7%A2%D7%95%D7%A9%D7%94-%D7%91%D7%97%D7%99%D7%99%D7%9D-%D7%90%D7%9C%D7%A2%D7%93-%D7%94%D7%93%D7%A8/?srsltid=AU7gw4WXOjq3WQM4Su8fXK_EPoNk0tx8JzLm41-LBfhUzGfyL3rG9lWn</t>
         </is>
       </c>
-      <c r="F136" t="inlineStr">
-        <is>
-          <t>0260505</t>
-        </is>
+      <c r="F136" t="n">
+        <v>260505</v>
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr"/>
@@ -4294,10 +4264,8 @@
           <t>http://makombalev.org.il/html5/dbMATENASIM.taf?DID=4469&amp;_0=%E2'%E0%E6</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr">
-        <is>
-          <t>0524539151</t>
-        </is>
+      <c r="F137" t="n">
+        <v>524539151</v>
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr"/>
@@ -4321,10 +4289,8 @@
           <t>https://nons.co.il/provider/%D7%99%D7%94%D7%9C%D7%95%D7%9D_%D7%A0%D7%99%D7%94%D7%95%D7%9C_%D7%95%D7%90%D7%97%D7%96%D7%A7%D7%94</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>0509870040</t>
-        </is>
+      <c r="F138" t="n">
+        <v>509870040</v>
       </c>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr"/>
@@ -4348,10 +4314,8 @@
           <t>https://www.medreviews.co.il/search/treatment/medical-management-by-nurse/sharon/kfar-yona</t>
         </is>
       </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>0554548554</t>
-        </is>
+      <c r="F139" t="n">
+        <v>554548554</v>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr"/>
@@ -4375,10 +4339,8 @@
           <t>https://hr.huji.ac.il/people/%D7%90%D7%95%D7%A8%D7%99-%D7%99%D7%A2%D7%A7%D7%91</t>
         </is>
       </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>025881085</t>
-        </is>
+      <c r="F140" t="n">
+        <v>25881085</v>
       </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr"/>
@@ -4402,10 +4364,8 @@
           <t>https://herzoglaw.co.il/he/our-team/yaakov-brandt/</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>0260713</t>
-        </is>
+      <c r="F141" t="n">
+        <v>260713</v>
       </c>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr"/>
@@ -4429,10 +4389,8 @@
           <t>https://www.mt-law.co.il/local/%D7%A2%D7%95%D7%A8%D7%9A-%D7%93%D7%99%D7%9F-%D7%A0%D7%99%D7%99%D7%93%D7%95%D7%AA-%D7%A1%D7%97%D7%A0%D7%99%D7%9F/</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr">
-        <is>
-          <t>0260326</t>
-        </is>
+      <c r="F142" t="n">
+        <v>260326</v>
       </c>
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr"/>
@@ -4456,10 +4414,8 @@
           <t>https://www.connectedbusinesses.co.il/job-offer/%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A4%D7%A8%D7%95%D7%99%D7%A7%D7%98%D7%99%D7%9D-%D7%94%D7%A0%D7%93%D7%A1%D7%99%D7%99%D7%9D-%D7%9E%D7%92%D7%99%D7%99%D7%A1%D7%AA-%D7%9E%D7%A0/</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t>0260616</t>
-        </is>
+      <c r="F143" t="n">
+        <v>260616</v>
       </c>
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr"/>
@@ -4483,10 +4439,8 @@
           <t>https://parkingtag.co.il/%D7%97%D7%91%D7%A8%D7%94-%D7%9C%D7%9E%D7%99%D7%9E%D7%95%D7%A9-%D7%96%D7%9B%D7%95%D7%99%D7%95%D7%AA/</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>0240814</t>
-        </is>
+      <c r="F144" t="n">
+        <v>240814</v>
       </c>
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr"/>
@@ -4510,10 +4464,8 @@
           <t>https://enp.co.il/projects/%D7%90%D7%95%D7%A4%D7%A7%D7%99%D7%9D-%D7%97%D7%91%D7%A8%D7%94-%D7%9E%D7%A0%D7%94%D7%9C%D7%AA-%D7%9C%D7%94%D7%A7%D7%9E%D7%94-%D7%95%D7%A4%D7%99%D7%AA%D7%95%D7%97-%D7%A9%D7%9B%D7%95%D7%A0%D7%AA-%D7%94/</t>
         </is>
       </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>00021024</t>
-        </is>
+      <c r="F145" t="n">
+        <v>21024</v>
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr"/>
@@ -4537,10 +4489,8 @@
           <t>https://www.mem.org.il/he/%D7%9E%D7%95%D7%A2%D7%A6%D7%94%D7%90%D7%96%D7%95%D7%A8/%D7%90%D7%95%D7%A4%D7%A7%D7%99%D7%9D?page=1</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>064266895223</t>
-        </is>
+      <c r="F146" t="n">
+        <v>64266895223</v>
       </c>
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr"/>
@@ -4564,10 +4514,8 @@
           <t>https://hadar-group.co.il/%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91%D7%A0%D7%99%D7%99%D7%A0%D7%99%D7%9D-%D7%A7%D7%98%D7%A0%D7%99%D7%9D-%D7%A4%D7%AA%D7%A8%D7%95%D7%9F-%D7%97%D7%9B%D7%9D-%D7%9C/</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t>0260318</t>
-        </is>
+      <c r="F147" t="n">
+        <v>260318</v>
       </c>
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr"/>
@@ -4591,10 +4539,8 @@
           <t>https://architecture.org.il/%D7%90%D7%99%D7%A0%D7%93%D7%A7%D7%A1/%D7%90%D7%97%D7%96%D7%A7%D7%AA-%D7%9E%D7%91%D7%A0%D7%99%D7%9D-%D7%A0%D7%99%D7%A7%D7%99%D7%95%D7%9F-%D7%95%D7%90%D7%91%D7%98%D7%97%D7%94-%D7%A1%D7%98%D7%A0%D7%9C%D7%99-%D7%A4%D7%A8%D7%99%D7%99%D7%A1/</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>0250417</t>
-        </is>
+      <c r="F148" t="n">
+        <v>250417</v>
       </c>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr"/>
@@ -4618,10 +4564,8 @@
           <t>https://www.centerteam.co.il/7-%D7%93%D7%91%D7%A8%D7%99%D7%9D-%D7%9C%D7%91%D7%93%D7%95%D7%A7-%D7%9C%D7%A4%D7%A0%D7%99-%D7%A9%D7%91%D7%95%D7%97%D7%A8%D7%99%D7%9D-%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%95%D7%A2/</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>0260224</t>
-        </is>
+      <c r="F149" t="n">
+        <v>260224</v>
       </c>
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr"/>
@@ -4668,10 +4612,8 @@
           <t>https://mt.haifa.ac.il/</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr">
-        <is>
-          <t>048288126</t>
-        </is>
+      <c r="F151" t="n">
+        <v>48288126</v>
       </c>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr"/>
@@ -4695,10 +4637,8 @@
           <t>https://www.rbsec.co.il/%D7%97%D7%91%D7%A8%D7%AA-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%9E%D7%91%D7%A0%D7%99%D7%9D</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr">
-        <is>
-          <t>035618888</t>
-        </is>
+      <c r="F152" t="n">
+        <v>35618888</v>
       </c>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr"/>
@@ -4722,10 +4662,8 @@
           <t>https://www.ocean-il.co.il/%D7%A9%D7%99%D7%A8%D7%95%D7%AA%D7%99-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%9E%D7%94%D7%90%D7%A8%D7%A5-%D7%95%D7%9E%D7%A8%D7%97%D7%95%D7%A7/</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr">
-        <is>
-          <t>010192625</t>
-        </is>
+      <c r="F153" t="n">
+        <v>10192625</v>
       </c>
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr"/>
@@ -4749,10 +4687,8 @@
           <t>https://kfgroup.co.il/%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%A0%D7%9B%D7%A1%D7%99%D7%9D-%D7%9B%D7%9C-%D7%9E%D7%94-%D7%A9%D7%A6%D7%A8%D7%99%D7%9A-%D7%9C%D7%93%D7%A2%D7%AA/</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr">
-        <is>
-          <t>0240827</t>
-        </is>
+      <c r="F154" t="n">
+        <v>240827</v>
       </c>
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr"/>
@@ -4776,10 +4712,8 @@
           <t>https://www.bedek-mivnim.co.il/%D7%90%D7%95%D7%93%D7%95%D7%AA.html</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr">
-        <is>
-          <t>071899861</t>
-        </is>
+      <c r="F155" t="n">
+        <v>71899861</v>
       </c>
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr"/>
@@ -4803,14 +4737,186 @@
           <t>https://mivnim.co.il/</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr">
-        <is>
-          <t>000040276453</t>
-        </is>
+      <c r="F156" t="n">
+        <v>40276453</v>
       </c>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr"/>
       <c r="I156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr"/>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>מסלול ניהול עסקי בכיר</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>ראשון לציון</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>info@lahav.ac.il</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>https://www.lahav.ac.il/program/%D7%9E%D7%A1%D7%9C%D7%95%D7%9C-%D7%A0%D7%99%D7%94%D7%95%D7%9C-%D7%91%D7%9B%D7%99%D7%A8/</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>0260526</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr"/>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>ד"ר בת חן נחמיאס בירן | הפקולטה להנדסה ע"ש איבי ואלדר פליישמן</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>בת ים</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>bathennb@tauex.tau.ac.il</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>https://engineering.tau.ac.il/profile/bathennb</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>05168198947</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr"/>
+      <c r="I158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr"/>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>הצהרת פרטיות תושבים מי רהט</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr"/>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>joseph.asaly18@gmail.com</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>https://www.m-rahat.co.il/prv2/</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>000421810168</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr"/>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>קבוצת יבנה</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr"/>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>office@thn.co.il</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>https://www.thn.co.il/testimonials1/%D7%A7%D7%91%D7%95%D7%A6%D7%AA-%D7%99%D7%91%D7%A0%D7%94/</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>000576981303</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr"/>
+      <c r="I160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr"/>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>חברות הקבוצה</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr"/>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>igorg@natoon-group.co.il</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>https://natoon-management.co.il/%D7%97%D7%91%D7%A8%D7%95%D7%AA-%D7%94%D7%A7%D7%91%D7%95%D7%A6%D7%94/</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>0171101</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr"/>
+      <c r="H161" t="inlineStr"/>
+      <c r="I161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr"/>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>פסגות ניהול מבנים: חברת ניהול מבנים בחיפה ובקריות</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>חיפה</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>psagot.clean@gmail.com</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>https://www.psagot-clean.co.il/</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>0772122602</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr"/>
+      <c r="I162" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>